<commit_message>
Update Net Income stat card and Revenue vs. Costs chart with new TTM data
</commit_message>
<xml_diff>
--- a/data/Business Overview - Stat Cards.xlsx
+++ b/data/Business Overview - Stat Cards.xlsx
@@ -1,37 +1,91 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaarkema/Documents/Strategic Planning/CD_StrategicPlanning/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92272E92-5F6A-CC43-96C4-6E15DDEC36BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="9880" yWindow="6220" windowWidth="20360" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Sub-label</t>
+  </si>
+  <si>
+    <t>TTM Jul 2026</t>
+  </si>
+  <si>
+    <t>TTM Jul 2025</t>
+  </si>
+  <si>
+    <t>TTM Jul 2026 (gal)</t>
+  </si>
+  <si>
+    <t>TTM Jul 2025 (gal)</t>
+  </si>
+  <si>
+    <t>Net Income</t>
+  </si>
+  <si>
+    <t>all sources</t>
+  </si>
+  <si>
+    <t>Milk Sold</t>
+  </si>
+  <si>
+    <t>hundredweight (cwt)</t>
+  </si>
+  <si>
+    <t>Milking Herd</t>
+  </si>
+  <si>
+    <t>average cows in milk</t>
+  </si>
+  <si>
+    <t>Cropland</t>
+  </si>
+  <si>
+    <t>owned &amp; rented acres</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,81 +104,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -412,117 +407,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="4" width="14" customWidth="1"/>
+    <col min="5" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-label</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>TTM Jul 2026</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TTM Jul 2025</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>TTM Jul 2026 (gal)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>TTM Jul 2025 (gal)</t>
-        </is>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Net Income</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>all sources</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>812573.5699999999</v>
-      </c>
-      <c r="D2" t="n">
-        <v>372712.98</v>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2">
+        <v>610096.01</v>
+      </c>
+      <c r="D2">
+        <v>324110.99</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Milk Sold</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>hundredweight (cwt)</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Milking Herd</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>average cows in milk</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4">
         <v>900</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cropland</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>owned &amp; rented acres</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>2500</v>
+      </c>
+      <c r="D5">
         <v>2500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Connect A2 status chart to real genetic-test data, wire milking herd headcount, smooth monthly production chart via day-rate normalization
</commit_message>
<xml_diff>
--- a/data/Business Overview - Stat Cards.xlsx
+++ b/data/Business Overview - Stat Cards.xlsx
@@ -1,91 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaarkema/Documents/Strategic Planning/CD_StrategicPlanning/data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92272E92-5F6A-CC43-96C4-6E15DDEC36BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9880" yWindow="6220" windowWidth="20360" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9880" yWindow="6220" windowWidth="20360" windowHeight="12240" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Sub-label</t>
-  </si>
-  <si>
-    <t>TTM Jul 2026</t>
-  </si>
-  <si>
-    <t>TTM Jul 2025</t>
-  </si>
-  <si>
-    <t>TTM Jul 2026 (gal)</t>
-  </si>
-  <si>
-    <t>TTM Jul 2025 (gal)</t>
-  </si>
-  <si>
-    <t>Net Income</t>
-  </si>
-  <si>
-    <t>all sources</t>
-  </si>
-  <si>
-    <t>Milk Sold</t>
-  </si>
-  <si>
-    <t>hundredweight (cwt)</t>
-  </si>
-  <si>
-    <t>Milking Herd</t>
-  </si>
-  <si>
-    <t>average cows in milk</t>
-  </si>
-  <si>
-    <t>Cropland</t>
-  </si>
-  <si>
-    <t>owned &amp; rented acres</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -104,22 +52,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -407,86 +414,118 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="4" width="14" customWidth="1"/>
-    <col min="5" max="6" width="20" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="4"/>
+    <col width="20" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TTM Jul 2026</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TTM Jul 2025</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TTM Jul 2026 (gal)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>TTM Jul 2025 (gal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>all sources</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>610096.01</v>
+      </c>
+      <c r="D2" t="n">
+        <v>324110.99</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Milk Sold</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>hundredweight (cwt)</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+      <c r="F3" t="n">
+        <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2">
-        <v>610096.01</v>
-      </c>
-      <c r="D2">
-        <v>324110.99</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Milking Herd</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>headcount, Aug 2026</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1226</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cropland</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>owned &amp; rented acres</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>2500</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>2500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Lbs/Cow/Day, Butterfat, SCC, and correct milking herd count from Casey's Aug 2026 notes; add footnote citations
</commit_message>
<xml_diff>
--- a/data/Business Overview - Stat Cards.xlsx
+++ b/data/Business Overview - Stat Cards.xlsx
@@ -504,11 +504,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>headcount, Aug 2026</t>
+          <t>headcount, Aug 2026 (milking only, excl. dry)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1226</v>
+        <v>1085</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1009</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Wire in Home page metrics that already have real data elsewhere
- Milk Sold stat card: 361,247 cwt (was ###), converted from Raw Milk
  Production's real Annual Production gallons figure
- Key Metrics at a Glance: Annual cwt, Lbs/Cow/Day, Butterfat %, and SCC
  now pull the same real numbers already shown on the Raw Milk Production
  page; Labor Hrs/cwt gets a real current-year weighted average from
  Monthly Operating Metrics (no reliable prior-year comparison yet, since
  that source only goes back to Jan '25)
- Utilization Rate and Crops yields stay ### - genuinely not tracked
  anywhere on the dashboard yet
- Sync data/Business Overview - Stat Cards.xlsx and data/Key Metrics at a
  Glance.xlsx to match

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Business Overview - Stat Cards.xlsx
+++ b/data/Business Overview - Stat Cards.xlsx
@@ -489,11 +489,17 @@
           <t>hundredweight (cwt)</t>
         </is>
       </c>
+      <c r="C3" t="n">
+        <v>361247</v>
+      </c>
+      <c r="D3" t="n">
+        <v>345778</v>
+      </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>4200548</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>4020672</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Confirm Key Metrics financials, add Annual Revenue card, drop two stat cards
- Un-grey the Financials rows in the Key Metrics at a Glance table now
  that TTM Ordinary Income/COGS/Expenses are confirmed; drop the
  "pending review" note.
- Add an Annual Revenue stat card to Home next to Net Income
  ($25,483,840, -2.3% YoY), relabel both cards' comparisons from TTM to
  Annual, and clarify in footnote 4 that the two cards use different
  income bases. Correct the underlying Business Overview - Stat Cards
  data file's stale Net Income figure ($610,096.01 -> $675,589) and add
  a Revenue row to it.
- Delete the "Total Value of Crops Produced" stat card from Crop
  Efficiency (and its now-unused footnote); renumber Crops Labor's
  footnote.
- Remove the "Benchmark $/Head" and "vs. Benchmark" columns from the
  Animal Sales Annual Summary table, and their now-orphaned footnote
  and source citations.
</commit_message>
<xml_diff>
--- a/data/Business Overview - Stat Cards.xlsx
+++ b/data/Business Overview - Stat Cards.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9880" yWindow="6220" windowWidth="20360" windowHeight="12240" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>610096.01</v>
+        <v>675589</v>
       </c>
       <c r="D2" t="n">
         <v>324110.99</v>
@@ -536,6 +536,24 @@
       </c>
       <c r="D5" t="n">
         <v>2500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ordinary income</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>25483840</v>
+      </c>
+      <c r="D6" t="n">
+        <v>26079541</v>
       </c>
     </row>
   </sheetData>

</xml_diff>